<commit_message>
Insurance Coverage + Hazard Data
</commit_message>
<xml_diff>
--- a/data/crop_data_france.xlsx
+++ b/data/crop_data_france.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arvedluetzen/Documents/Coding-Projects/mus-climada/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD17C485-3747-2447-A356-73A24421479A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38E86C50-023C-EF4B-A11F-34E5B39F287F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="22780" windowHeight="14540" xr2:uid="{0438FC33-3D89-4307-AEAA-96EE8E74AC4E}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{0438FC33-3D89-4307-AEAA-96EE8E74AC4E}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="202">
   <si>
     <t>number_department</t>
   </si>
@@ -639,6 +639,9 @@
   </si>
   <si>
     <t>value</t>
+  </si>
+  <si>
+    <t>insurance</t>
   </si>
 </sst>
 </file>
@@ -686,11 +689,11 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -818,9 +821,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -842,6 +842,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1201,6 +1204,9 @@
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="E1" s="23" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
@@ -1215,6 +1221,9 @@
       <c r="D2" s="6">
         <v>5762.4</v>
       </c>
+      <c r="E2">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="3" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
@@ -1228,6 +1237,9 @@
       </c>
       <c r="D3" s="8">
         <v>7361.7</v>
+      </c>
+      <c r="E3">
+        <v>0.32</v>
       </c>
       <c r="F3" s="9"/>
       <c r="G3" s="9"/>
@@ -1249,6 +1261,9 @@
       <c r="D4" s="8">
         <v>7340.1</v>
       </c>
+      <c r="E4">
+        <v>0.3</v>
+      </c>
       <c r="F4" s="9"/>
       <c r="G4" s="9"/>
       <c r="H4" s="9"/>
@@ -1269,6 +1284,9 @@
       <c r="D5" s="8">
         <v>6925.2</v>
       </c>
+      <c r="E5">
+        <v>0.18</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
@@ -1283,6 +1301,9 @@
       <c r="D6" s="8">
         <v>5548.7</v>
       </c>
+      <c r="E6">
+        <v>0.18</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
@@ -1297,6 +1318,9 @@
       <c r="D7" s="8">
         <v>4298.6000000000004</v>
       </c>
+      <c r="E7">
+        <v>0.18</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
@@ -1310,6 +1334,9 @@
       </c>
       <c r="D8" s="8">
         <v>5528.6</v>
+      </c>
+      <c r="E8">
+        <v>0.3</v>
       </c>
       <c r="F8" s="10"/>
       <c r="G8" s="10"/>
@@ -1330,6 +1357,9 @@
       <c r="D9" s="8">
         <v>5229.3999999999996</v>
       </c>
+      <c r="E9">
+        <v>0.42</v>
+      </c>
       <c r="F9" s="11"/>
       <c r="G9" s="11"/>
       <c r="H9" s="11"/>
@@ -1349,6 +1379,9 @@
       <c r="D10" s="8">
         <v>4889.8999999999996</v>
       </c>
+      <c r="E10">
+        <v>0.4</v>
+      </c>
       <c r="F10" s="12"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
@@ -1364,6 +1397,9 @@
       <c r="D11" s="8">
         <v>6004.2</v>
       </c>
+      <c r="E11">
+        <v>0.42</v>
+      </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
@@ -1378,6 +1414,9 @@
       <c r="D12" s="8">
         <v>6139</v>
       </c>
+      <c r="E12">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
@@ -1391,6 +1430,9 @@
       </c>
       <c r="D13" s="8">
         <v>8735.1</v>
+      </c>
+      <c r="E13">
+        <v>0.4</v>
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
@@ -1410,6 +1452,9 @@
       <c r="D14" s="8">
         <v>5087.5</v>
       </c>
+      <c r="E14">
+        <v>0.18</v>
+      </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
@@ -1424,6 +1469,9 @@
       <c r="D15" s="8">
         <v>5534.5</v>
       </c>
+      <c r="E15">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
@@ -1437,6 +1485,9 @@
       </c>
       <c r="D16" s="8">
         <v>5726</v>
+      </c>
+      <c r="E16">
+        <v>0.3</v>
       </c>
       <c r="F16" s="14"/>
       <c r="G16" s="14"/>
@@ -1444,7 +1495,7 @@
       <c r="I16" s="14"/>
       <c r="J16" s="14"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
         <v>33</v>
       </c>
@@ -1457,8 +1508,11 @@
       <c r="D17" s="8">
         <v>5956</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E17">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
         <v>35</v>
       </c>
@@ -1471,8 +1525,11 @@
       <c r="D18" s="8">
         <v>6863.8</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E18">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
         <v>37</v>
       </c>
@@ -1485,8 +1542,11 @@
       <c r="D19" s="8">
         <v>7235</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E19">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
         <v>39</v>
       </c>
@@ -1499,8 +1559,11 @@
       <c r="D20" s="8">
         <v>5856.8</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E20">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
         <v>41</v>
       </c>
@@ -1513,8 +1576,11 @@
       <c r="D21" s="8">
         <v>4014.2</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E21">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
         <v>43</v>
       </c>
@@ -1527,8 +1593,11 @@
       <c r="D22" s="8">
         <v>4665.6000000000004</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E22">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
         <v>45</v>
       </c>
@@ -1541,8 +1610,11 @@
       <c r="D23" s="8">
         <v>8763.2000000000007</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E23">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
         <v>47</v>
       </c>
@@ -1555,8 +1627,11 @@
       <c r="D24" s="8">
         <v>6877.6</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E24">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
         <v>49</v>
       </c>
@@ -1569,8 +1644,11 @@
       <c r="D25" s="8">
         <v>5565.4</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E25">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
         <v>51</v>
       </c>
@@ -1583,8 +1661,11 @@
       <c r="D26" s="8">
         <v>9060</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E26">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>53</v>
       </c>
@@ -1597,8 +1678,11 @@
       <c r="D27" s="8">
         <v>5232.6000000000004</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E27">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
         <v>55</v>
       </c>
@@ -1611,8 +1695,11 @@
       <c r="D28" s="8">
         <v>6530</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E28">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
         <v>57</v>
       </c>
@@ -1625,8 +1712,11 @@
       <c r="D29" s="8">
         <v>6039.9</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E29">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
         <v>59</v>
       </c>
@@ -1640,7 +1730,7 @@
         <v>5880</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
         <v>61</v>
       </c>
@@ -1654,7 +1744,7 @@
         <v>6733</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
         <v>63</v>
       </c>
@@ -1666,6 +1756,9 @@
       </c>
       <c r="D32" s="8">
         <v>5852.8</v>
+      </c>
+      <c r="E32">
+        <v>0.4</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -1681,6 +1774,9 @@
       <c r="D33" s="8">
         <v>6309.3</v>
       </c>
+      <c r="E33">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
@@ -1695,7 +1791,9 @@
       <c r="D34" s="8">
         <v>6256.8</v>
       </c>
-      <c r="E34" s="15"/>
+      <c r="E34">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
@@ -1710,6 +1808,9 @@
       <c r="D35" s="8">
         <v>9975.6</v>
       </c>
+      <c r="E35">
+        <v>0.39</v>
+      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
@@ -1724,6 +1825,9 @@
       <c r="D36" s="8">
         <v>6101</v>
       </c>
+      <c r="E36">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
@@ -1738,6 +1842,9 @@
       <c r="D37" s="8">
         <v>6774.7</v>
       </c>
+      <c r="E37">
+        <v>0.02</v>
+      </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
@@ -1752,6 +1859,9 @@
       <c r="D38" s="8">
         <v>6790.6</v>
       </c>
+      <c r="E38">
+        <v>0.45</v>
+      </c>
     </row>
     <row r="39" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
@@ -1766,6 +1876,9 @@
       <c r="D39" s="8">
         <v>6126.7</v>
       </c>
+      <c r="E39">
+        <v>0.45</v>
+      </c>
     </row>
     <row r="40" spans="1:5" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
@@ -1780,6 +1893,9 @@
       <c r="D40" s="8">
         <v>7431.5</v>
       </c>
+      <c r="E40">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="41" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
@@ -1794,6 +1910,9 @@
       <c r="D41" s="8">
         <v>4999.2</v>
       </c>
+      <c r="E41">
+        <v>0.36</v>
+      </c>
     </row>
     <row r="42" spans="1:5" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
@@ -1808,6 +1927,9 @@
       <c r="D42" s="8">
         <v>9242.6</v>
       </c>
+      <c r="E42">
+        <v>0.39</v>
+      </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
@@ -1822,6 +1944,9 @@
       <c r="D43" s="8">
         <v>6343.4</v>
       </c>
+      <c r="E43">
+        <v>0.45</v>
+      </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" s="7" t="s">
@@ -1836,6 +1961,9 @@
       <c r="D44" s="8">
         <v>4780.6000000000004</v>
       </c>
+      <c r="E44">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
@@ -1850,6 +1978,9 @@
       <c r="D45" s="8">
         <v>4977.1000000000004</v>
       </c>
+      <c r="E45">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
@@ -1864,6 +1995,9 @@
       <c r="D46" s="8">
         <v>6874.4</v>
       </c>
+      <c r="E46">
+        <v>0.16</v>
+      </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
@@ -1878,6 +2012,9 @@
       <c r="D47" s="8">
         <v>6775.2</v>
       </c>
+      <c r="E47">
+        <v>0.45</v>
+      </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" s="7" t="s">
@@ -1892,8 +2029,11 @@
       <c r="D48" s="8">
         <v>5216.5</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E48">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
         <v>97</v>
       </c>
@@ -1906,8 +2046,11 @@
       <c r="D49" s="8">
         <v>5360.9</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E49">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
         <v>99</v>
       </c>
@@ -1920,8 +2063,11 @@
       <c r="D50" s="8">
         <v>5166.8999999999996</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E50">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
         <v>101</v>
       </c>
@@ -1934,8 +2080,11 @@
       <c r="D51" s="8">
         <v>7106.6</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E51">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
         <v>103</v>
       </c>
@@ -1948,8 +2097,11 @@
       <c r="D52" s="8">
         <v>5951.5</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E52">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
         <v>105</v>
       </c>
@@ -1962,8 +2114,11 @@
       <c r="D53" s="8">
         <v>8169.1</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E53">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
         <v>107</v>
       </c>
@@ -1976,8 +2131,11 @@
       <c r="D54" s="8">
         <v>6210.6</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E54">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
         <v>109</v>
       </c>
@@ -1990,8 +2148,11 @@
       <c r="D55" s="8">
         <v>5175.2</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E55">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
         <v>111</v>
       </c>
@@ -2004,8 +2165,11 @@
       <c r="D56" s="8">
         <v>5245.9</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E56">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
         <v>113</v>
       </c>
@@ -2018,8 +2182,11 @@
       <c r="D57" s="8">
         <v>6211.4</v>
       </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E57">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
         <v>115</v>
       </c>
@@ -2032,8 +2199,11 @@
       <c r="D58" s="8">
         <v>6822.6</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E58">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" s="7" t="s">
         <v>117</v>
       </c>
@@ -2046,8 +2216,11 @@
       <c r="D59" s="8">
         <v>6216.3</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E59">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="s">
         <v>119</v>
       </c>
@@ -2060,8 +2233,11 @@
       <c r="D60" s="8">
         <v>6816.7</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E60">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
         <v>121</v>
       </c>
@@ -2074,8 +2250,11 @@
       <c r="D61" s="8">
         <v>5742.8</v>
       </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E61">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
         <v>123</v>
       </c>
@@ -2088,8 +2267,11 @@
       <c r="D62" s="8">
         <v>5860.2</v>
       </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E62">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
         <v>125</v>
       </c>
@@ -2102,8 +2284,11 @@
       <c r="D63" s="8">
         <v>6103.4</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E63">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
         <v>127</v>
       </c>
@@ -2116,8 +2301,11 @@
       <c r="D64" s="8">
         <v>6671.4</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E64">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
         <v>129</v>
       </c>
@@ -2130,8 +2318,11 @@
       <c r="D65" s="8">
         <v>7969.7</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E65">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" s="7" t="s">
         <v>131</v>
       </c>
@@ -2144,8 +2335,11 @@
       <c r="D66" s="8">
         <v>7644.8</v>
       </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E66">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
         <v>133</v>
       </c>
@@ -2158,8 +2352,11 @@
       <c r="D67" s="8">
         <v>4464</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E67">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68" s="7" t="s">
         <v>135</v>
       </c>
@@ -2172,8 +2369,11 @@
       <c r="D68" s="8">
         <v>4116</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E68">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="s">
         <v>137</v>
       </c>
@@ -2186,8 +2386,11 @@
       <c r="D69" s="8">
         <v>4755</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E69">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70" s="7" t="s">
         <v>139</v>
       </c>
@@ -2200,8 +2403,11 @@
       <c r="D70" s="8">
         <v>3525.2</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E70">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71" s="7" t="s">
         <v>141</v>
       </c>
@@ -2214,8 +2420,11 @@
       <c r="D71" s="8">
         <v>3249.1</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E71">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" s="7" t="s">
         <v>143</v>
       </c>
@@ -2228,8 +2437,11 @@
       <c r="D72" s="8">
         <v>5360.1</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E72">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
         <v>145</v>
       </c>
@@ -2242,8 +2454,11 @@
       <c r="D73" s="8">
         <v>8574.7000000000007</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E73">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" s="7" t="s">
         <v>147</v>
       </c>
@@ -2256,8 +2471,11 @@
       <c r="D74" s="8">
         <v>6206</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E74">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
         <v>149</v>
       </c>
@@ -2270,8 +2488,11 @@
       <c r="D75" s="8">
         <v>6028.3</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E75">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="s">
         <v>151</v>
       </c>
@@ -2284,8 +2505,11 @@
       <c r="D76" s="8">
         <v>4387.8</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E76">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" s="7" t="s">
         <v>153</v>
       </c>
@@ -2298,8 +2522,11 @@
       <c r="D77" s="8">
         <v>105.4</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E77">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" s="7" t="s">
         <v>155</v>
       </c>
@@ -2312,8 +2539,11 @@
       <c r="D78" s="8">
         <v>6277.6</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E78">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" s="7" t="s">
         <v>157</v>
       </c>
@@ -2326,8 +2556,11 @@
       <c r="D79" s="8">
         <v>5915.3</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E79">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" s="7" t="s">
         <v>159</v>
       </c>
@@ -2340,8 +2573,11 @@
       <c r="D80" s="8">
         <v>2284.4</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E80">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" s="7" t="s">
         <v>161</v>
       </c>
@@ -2354,8 +2590,11 @@
       <c r="D81" s="8">
         <v>5999.4</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E81">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" s="7" t="s">
         <v>163</v>
       </c>
@@ -2368,8 +2607,11 @@
       <c r="D82" s="8">
         <v>6170.1</v>
       </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E82">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" s="7" t="s">
         <v>165</v>
       </c>
@@ -2382,8 +2624,11 @@
       <c r="D83" s="8">
         <v>5757.9</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E83">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84" s="7" t="s">
         <v>167</v>
       </c>
@@ -2396,8 +2641,11 @@
       <c r="D84" s="8">
         <v>3718.3</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E84">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85" s="7" t="s">
         <v>169</v>
       </c>
@@ -2410,8 +2658,11 @@
       <c r="D85" s="8">
         <v>5972.5</v>
       </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E85">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86" s="7" t="s">
         <v>171</v>
       </c>
@@ -2424,8 +2675,11 @@
       <c r="D86" s="8">
         <v>3567.3</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E86">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87" s="7" t="s">
         <v>173</v>
       </c>
@@ -2438,8 +2692,11 @@
       <c r="D87" s="8">
         <v>6719.6</v>
       </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E87">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88" s="7" t="s">
         <v>175</v>
       </c>
@@ -2452,8 +2709,11 @@
       <c r="D88" s="8">
         <v>6990.4</v>
       </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E88">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89" s="7" t="s">
         <v>177</v>
       </c>
@@ -2466,8 +2726,11 @@
       <c r="D89" s="8">
         <v>5520.1</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E89">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90" s="7" t="s">
         <v>179</v>
       </c>
@@ -2480,8 +2743,11 @@
       <c r="D90" s="8">
         <v>5873.8</v>
       </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E90">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" s="7" t="s">
         <v>181</v>
       </c>
@@ -2494,8 +2760,11 @@
       <c r="D91" s="8">
         <v>7427.4</v>
       </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E91">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92" s="7" t="s">
         <v>183</v>
       </c>
@@ -2508,8 +2777,11 @@
       <c r="D92" s="8">
         <v>609.4</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E92">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" s="7" t="s">
         <v>185</v>
       </c>
@@ -2522,36 +2794,45 @@
       <c r="D93" s="8">
         <v>1804.4</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E93">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" s="7" t="s">
         <v>187</v>
       </c>
       <c r="B94" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="C94" s="16" t="s">
+      <c r="C94" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="D94" s="16">
+      <c r="D94" s="15">
         <v>175.6</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E94">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95" s="7" t="s">
         <v>190</v>
       </c>
       <c r="B95" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="C95" s="16" t="s">
+      <c r="C95" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="D95" s="16">
+      <c r="D95" s="15">
         <v>236.2</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E95">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96" s="7" t="s">
         <v>192</v>
       </c>
@@ -2564,45 +2845,51 @@
       <c r="D96" s="8">
         <v>245</v>
       </c>
+      <c r="E96">
+        <v>0.72</v>
+      </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A97" s="17" t="s">
+      <c r="A97" s="16" t="s">
         <v>194</v>
       </c>
-      <c r="B97" s="17" t="s">
+      <c r="B97" s="16" t="s">
         <v>195</v>
       </c>
-      <c r="C97" s="18">
+      <c r="C97" s="17">
         <v>38.1</v>
       </c>
-      <c r="D97" s="18">
+      <c r="D97" s="17">
         <v>1245.9000000000001</v>
       </c>
+      <c r="E97">
+        <v>0.72</v>
+      </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A98" s="19" t="s">
+      <c r="A98" s="18" t="s">
         <v>196</v>
       </c>
-      <c r="D98" s="20"/>
+      <c r="D98" s="19"/>
     </row>
     <row r="99" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A99" s="23" t="s">
+      <c r="A99" s="22" t="s">
         <v>197</v>
       </c>
-      <c r="B99" s="23"/>
-      <c r="C99" s="23"/>
-      <c r="D99" s="21"/>
-      <c r="E99" s="21"/>
-      <c r="F99" s="21"/>
-      <c r="G99" s="21"/>
+      <c r="B99" s="22"/>
+      <c r="C99" s="22"/>
+      <c r="D99" s="20"/>
+      <c r="E99" s="20"/>
+      <c r="F99" s="20"/>
+      <c r="G99" s="20"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A100" s="22" t="s">
+      <c r="A100" s="21" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A101" s="22" t="s">
+      <c r="A101" s="21" t="s">
         <v>199</v>
       </c>
     </row>

</xml_diff>